<commit_message>
Used excel utils for login
</commit_message>
<xml_diff>
--- a/src/test/resources/BookingData.xlsx
+++ b/src/test/resources/BookingData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2492243_cognizant_com/Documents/Desktop/cinebook-self/Testing_CineBook/src/test/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Testing_Cinebook\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_F25DC773A252ABDACC104862791E56B65ADE58FA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8193C8EC-256B-4256-9E96-75D4730F6BDF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF3C11A-B09D-4E42-8986-6AC5DEF94BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1300" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="shows" sheetId="1" r:id="rId1"/>
@@ -33,10 +33,10 @@
     <t>show-id</t>
   </si>
   <si>
-    <t>movie-book-3</t>
+    <t>movie-book-1</t>
   </si>
   <si>
-    <t>show-12</t>
+    <t>show-1</t>
   </si>
 </sst>
 </file>
@@ -89,10 +89,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>